<commit_message>
refactor: merge vendor and keyword tabs into unified vendor management tab
</commit_message>
<xml_diff>
--- a/data/target_form/강화군농협.xlsx
+++ b/data/target_form/강화군농협.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/ae7f7f815e37025b/문서/365건강농산/목표양식/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\skawl\PycharmProjects\365배포\data\target_form\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="14" documentId="13_ncr:1_{6861D042-D17B-4809-96AE-9B2F5A9AD1AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0F13291E-2C3E-48FD-907E-EEA9A17455B1}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E2EA390-66C6-4ABB-A768-EBC9A84C0B33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="0" windowWidth="12980" windowHeight="16090" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="16220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="24">
   <si>
     <t>수량</t>
   </si>
@@ -62,14 +62,6 @@
   </si>
   <si>
     <t>택배사코드(필수)</t>
-  </si>
-  <si>
-    <t>수신: 강화군 농협</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>발신: 365건강농산</t>
-    <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
     <t>100292</t>
@@ -118,7 +110,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -138,21 +130,6 @@
       <charset val="129"/>
     </font>
     <font>
-      <sz val="20"/>
-      <color rgb="FF000000"/>
-      <name val="맑은 고딕"/>
-      <family val="3"/>
-      <charset val="129"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color rgb="FF000000"/>
-      <name val="맑은 고딕"/>
-      <family val="3"/>
-      <charset val="129"/>
-    </font>
-    <font>
       <b/>
       <sz val="9"/>
       <color rgb="FFFFFFFF"/>
@@ -160,14 +137,6 @@
       <family val="3"/>
       <charset val="129"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="22"/>
-      <color rgb="FF000000"/>
-      <name val="맑은 고딕"/>
-      <family val="3"/>
-      <charset val="129"/>
     </font>
     <font>
       <b/>
@@ -206,7 +175,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -229,24 +198,6 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
@@ -256,7 +207,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -269,26 +220,17 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -306,10 +248,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -602,7 +540,7 @@
   <sheetPr codeName="1">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:Q3"/>
+  <dimension ref="A1:Q2"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="12.9140625" style="1" bestFit="1" customWidth="1"/>
@@ -624,120 +562,101 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="24" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B1" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="C1" s="9"/>
-      <c r="D1" s="9"/>
-      <c r="E1" s="9"/>
-      <c r="F1" s="9"/>
-      <c r="G1" s="9"/>
-      <c r="H1" s="9"/>
-      <c r="L1" s="10" t="s">
-        <v>13</v>
-      </c>
-      <c r="M1" s="10"/>
+      <c r="A1" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="H1" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="I1" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="J1" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="K1" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="L1" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="M1" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="N1" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="O1" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="P1" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="Q1" s="4" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="2" spans="1:17" ht="17.25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A2" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="C2" s="4" t="s">
+      <c r="B2" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="D2" s="6">
+        <v>1</v>
+      </c>
+      <c r="E2" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="F2" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="G2" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="H2" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="D2" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="F2" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="G2" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="H2" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="I2" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="J2" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="K2" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="L2" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="M2" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="N2" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="O2" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="P2" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="Q2" s="4" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="3" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B3" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="C3" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="D3" s="6">
-        <v>1</v>
-      </c>
-      <c r="E3" s="6" t="s">
+      <c r="I2" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="F3" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="G3" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="H3" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="I3" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="J3" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="K3" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="L3" s="6"/>
-      <c r="M3" s="7">
+      <c r="J2" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="K2" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="L2" s="6"/>
+      <c r="M2" s="7">
         <v>2149040229</v>
       </c>
-      <c r="N3" s="6"/>
-      <c r="O3" s="6"/>
-      <c r="P3" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="Q3" s="6"/>
+      <c r="N2" s="6"/>
+      <c r="O2" s="6"/>
+      <c r="P2" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q2" s="6"/>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="B1:H1"/>
-    <mergeCell ref="L1:M1"/>
-  </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.69972223043441772" right="0.69972223043441772" top="0.75" bottom="0.75" header="0.30000001192092896" footer="0.30000001192092896"/>
   <pageSetup paperSize="9" scale="79" orientation="landscape" r:id="rId1"/>

</xml_diff>

<commit_message>
auto: upload form 강화군농협.xlsx
</commit_message>
<xml_diff>
--- a/data/target_form/강화군농협.xlsx
+++ b/data/target_form/강화군농협.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24228"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\skawl\PycharmProjects\365배포\data\target_form\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\365건강\Desktop\사방넷발주\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E2EA390-66C6-4ABB-A768-EBC9A84C0B33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C925062-AE8D-44DF-BDF1-C6744F7FEDD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="16220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1" sheetId="1" r:id="rId1"/>
@@ -26,20 +26,32 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="27">
   <si>
     <t>수량</t>
   </si>
   <si>
+    <t>수령인 전화번호</t>
+  </si>
+  <si>
     <t>수령인 휴대폰</t>
   </si>
   <si>
     <t>우편번호</t>
   </si>
   <si>
+    <t>수령인</t>
+  </si>
+  <si>
     <t>구매자</t>
   </si>
   <si>
+    <t>주문번호(쇼핑몰)</t>
+  </si>
+  <si>
+    <t>상품약어</t>
+  </si>
+  <si>
     <t>수령인주소</t>
   </si>
   <si>
@@ -52,6 +64,9 @@
     <t>.</t>
   </si>
   <si>
+    <t>사방넷 주문번호(필수)</t>
+  </si>
+  <si>
     <t>송장번호(필수)</t>
   </si>
   <si>
@@ -64,53 +79,43 @@
     <t>택배사코드(필수)</t>
   </si>
   <si>
+    <t>수신: 강화군 농협</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>발신: 365건강농산</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
     <t>100292</t>
   </si>
   <si>
-    <t>010-2542-4208</t>
-  </si>
-  <si>
-    <t>김화영</t>
-  </si>
-  <si>
-    <t>문앞에두고가세요</t>
-  </si>
-  <si>
-    <t>596-36</t>
+    <t>01022577235</t>
+  </si>
+  <si>
+    <t>김형국</t>
+  </si>
+  <si>
+    <t>[고객배송메모]부재 시 문 앞에 놓아주세요.</t>
+  </si>
+  <si>
+    <t>[063-54] 서울특별시 강남구 광평로31길 27 (삼성아파트)  102동 101호</t>
+  </si>
+  <si>
+    <t>063-54</t>
+  </si>
+  <si>
+    <t>010-2257-7235</t>
   </si>
   <si>
     <t>강화군농협 고시히카리 쌀10kg</t>
-  </si>
-  <si>
-    <t>사방넷 주문번호(필수)</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>주문번호(쇼핑몰)</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>수령인</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>상품약어</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>수령인 전화번호</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>[596-36] 전라남도 여수시 덕양로 157 (화장동, 주공3단지아파트) 304동105호</t>
-    <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -126,6 +131,21 @@
     <font>
       <sz val="8"/>
       <name val="돋움"/>
+      <family val="3"/>
+      <charset val="129"/>
+    </font>
+    <font>
+      <sz val="20"/>
+      <color rgb="FF000000"/>
+      <name val="맑은 고딕"/>
+      <family val="3"/>
+      <charset val="129"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color rgb="FF000000"/>
+      <name val="맑은 고딕"/>
       <family val="3"/>
       <charset val="129"/>
     </font>
@@ -137,6 +157,14 @@
       <family val="3"/>
       <charset val="129"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="22"/>
+      <color rgb="FF000000"/>
+      <name val="맑은 고딕"/>
+      <family val="3"/>
+      <charset val="129"/>
     </font>
     <font>
       <b/>
@@ -175,7 +203,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -198,6 +226,24 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
@@ -207,7 +253,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -220,16 +266,25 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -540,123 +595,141 @@
   <sheetPr codeName="1">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:Q2"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.45"/>
+  <dimension ref="A1:Q3"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12.9140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.75" style="1" customWidth="1"/>
+    <col min="2" max="2" width="11" style="1" customWidth="1"/>
     <col min="3" max="3" width="33.75" style="2" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="4.75" style="3" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="13.58203125" style="2" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.08203125" style="2" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="39.9140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.83203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="13.625" style="2" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.125" style="2" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="40" style="2" customWidth="1"/>
+    <col min="9" max="9" width="9.875" style="3" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="7.25" style="2" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="12.25" style="2" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="12.08203125" style="2" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="16.6640625" style="2" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="10.58203125" style="2" customWidth="1"/>
-    <col min="15" max="15" width="10.08203125" style="1" customWidth="1"/>
-    <col min="16" max="17" width="12.9140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="18" max="16384" width="9" style="1"/>
+    <col min="12" max="12" width="12.125" style="2" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="9" style="2"/>
+    <col min="14" max="14" width="10.625" style="2" customWidth="1"/>
+    <col min="15" max="15" width="10.125" style="1" customWidth="1"/>
+    <col min="16" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" ht="24" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A1" s="4" t="s">
+    <row r="1" spans="1:17" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B1" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1" s="7"/>
+      <c r="D1" s="7"/>
+      <c r="E1" s="7"/>
+      <c r="F1" s="7"/>
+      <c r="G1" s="7"/>
+      <c r="H1" s="7"/>
+      <c r="L1" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="M1" s="8"/>
+    </row>
+    <row r="2" spans="1:17" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="J2" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="K2" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="L2" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="M2" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="N2" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="O2" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="P2" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q2" s="4" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="3" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B3" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="C3" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="D3" s="9">
+        <v>1</v>
+      </c>
+      <c r="E3" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="F3" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="G3" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="H3" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="I3" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="J3" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="K3" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="L3" s="9"/>
+      <c r="M3" s="10">
+        <v>2158017237</v>
+      </c>
+      <c r="N3" s="9"/>
+      <c r="O3" s="9"/>
+      <c r="P3" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="B1" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="F1" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="G1" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="H1" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="I1" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="J1" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="K1" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="L1" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="M1" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="N1" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="O1" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="P1" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="Q1" s="4" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="2" spans="1:17" ht="17.25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B2" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="C2" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="D2" s="6">
-        <v>1</v>
-      </c>
-      <c r="E2" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="F2" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="G2" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="H2" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="I2" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="J2" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="K2" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="L2" s="6"/>
-      <c r="M2" s="7">
-        <v>2149040229</v>
-      </c>
-      <c r="N2" s="6"/>
-      <c r="O2" s="6"/>
-      <c r="P2" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="Q2" s="6"/>
+      <c r="Q3" s="9"/>
     </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B1:H1"/>
+    <mergeCell ref="L1:M1"/>
+  </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.69972223043441772" right="0.69972223043441772" top="0.75" bottom="0.75" header="0.30000001192092896" footer="0.30000001192092896"/>
   <pageSetup paperSize="9" scale="79" orientation="landscape" r:id="rId1"/>
@@ -667,7 +740,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="17" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <sheetData/>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.69972223043441772" right="0.69972223043441772" top="0.75" bottom="0.75" header="0.30000001192092896" footer="0.30000001192092896"/>
@@ -679,7 +752,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="17" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <sheetData/>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.69972223043441772" right="0.69972223043441772" top="0.75" bottom="0.75" header="0.30000001192092896" footer="0.30000001192092896"/>
@@ -691,7 +764,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <sheetPr codeName="Sheet3"/>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="17" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <sheetData/>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.74805557727813721" right="0.74805557727813721" top="0.98430556058883667" bottom="0.98430556058883667" header="0.51138889789581299" footer="0.51138889789581299"/>

</xml_diff>